<commit_message>
Update experimental design status
</commit_message>
<xml_diff>
--- a/DATA/DISENO_EXPERIMENTAL/catalogo_experimentos.xlsx
+++ b/DATA/DISENO_EXPERIMENTAL/catalogo_experimentos.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,16 +16,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +33,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,24 +41,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -429,52 +416,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Experimento</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Dominio</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Pregunta_Investigacion</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Objetivo_Experimento</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Variable_Objetivo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tipo_Problema</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Ventana</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Horizonte</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -668,7 +655,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Ejecutado</t>
         </is>
       </c>
     </row>
@@ -865,6 +852,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>